<commit_message>
finished keyboard emulator circuit and some BOMs
</commit_message>
<xml_diff>
--- a/keyboard_emulator/BOM.xlsx
+++ b/keyboard_emulator/BOM.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -41,6 +41,21 @@
   </si>
   <si>
     <t xml:space="preserve">Store</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PCB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arduino Pro Micro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pin Headers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spring Terminal – 4Pin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Push Button</t>
   </si>
   <si>
     <t xml:space="preserve">**</t>
@@ -72,7 +87,6 @@
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -95,14 +109,12 @@
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="0"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="0"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -400,7 +412,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G1048576"/>
   <sheetFormatPr defaultColWidth="10.55078125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
@@ -439,12 +451,18 @@
       <c r="A2" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="5"/>
+      <c r="B2" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="7" t="n">
+        <v>150</v>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="E2" s="8" t="n">
         <f aca="false">C2*D2</f>
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="F2" s="9"/>
       <c r="G2" s="10"/>
@@ -453,12 +471,18 @@
       <c r="A3" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="5"/>
+      <c r="B3" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="7" t="n">
+        <v>475</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="E3" s="8" t="n">
         <f aca="false">C3*D3</f>
-        <v>0</v>
+        <v>475</v>
       </c>
       <c r="F3" s="9"/>
       <c r="G3" s="10"/>
@@ -467,12 +491,18 @@
       <c r="A4" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="6"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="5"/>
+      <c r="B4" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>2</v>
+      </c>
       <c r="E4" s="8" t="n">
         <f aca="false">C4*D4</f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F4" s="9"/>
       <c r="G4" s="10"/>
@@ -481,12 +511,18 @@
       <c r="A5" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="6"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="5"/>
+      <c r="B5" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>2</v>
+      </c>
       <c r="E5" s="8" t="n">
         <f aca="false">C5*D5</f>
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F5" s="9"/>
       <c r="G5" s="10"/>
@@ -495,138 +531,105 @@
       <c r="A6" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="6"/>
-      <c r="C6" s="7"/>
-      <c r="D6" s="5"/>
+      <c r="B6" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>4</v>
+      </c>
       <c r="E6" s="8" t="n">
         <f aca="false">C6*D6</f>
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="F6" s="9"/>
       <c r="G6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="n">
-        <v>6</v>
-      </c>
+      <c r="A7" s="5"/>
       <c r="B7" s="6"/>
       <c r="C7" s="7"/>
       <c r="D7" s="5"/>
-      <c r="E7" s="8" t="n">
-        <f aca="false">C7*D7</f>
-        <v>0</v>
-      </c>
+      <c r="E7" s="8"/>
       <c r="F7" s="9"/>
       <c r="G7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="6"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="5"/>
+      <c r="A8" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>70</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>2</v>
+      </c>
       <c r="E8" s="8" t="n">
         <f aca="false">C8*D8</f>
-        <v>0</v>
+        <v>140</v>
       </c>
       <c r="F8" s="9"/>
       <c r="G8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="n">
-        <v>8</v>
-      </c>
+      <c r="A9" s="5"/>
       <c r="B9" s="6"/>
       <c r="C9" s="7"/>
       <c r="D9" s="5"/>
-      <c r="E9" s="8" t="n">
-        <f aca="false">C9*D9</f>
-        <v>0</v>
-      </c>
-      <c r="F9" s="9"/>
+      <c r="E9" s="8"/>
       <c r="G9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5"/>
-      <c r="B10" s="6"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="8"/>
+      <c r="A10" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="13" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D10" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="14" t="n">
+        <f aca="false">C10*D10</f>
+        <v>2000</v>
+      </c>
       <c r="F10" s="9"/>
       <c r="G10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C11" s="7" t="n">
-        <v>70</v>
-      </c>
-      <c r="D11" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" s="8" t="n">
-        <f aca="false">C11*D11</f>
-        <v>70</v>
-      </c>
+      <c r="A11" s="5"/>
+      <c r="B11" s="15"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="18"/>
       <c r="F11" s="9"/>
       <c r="G11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5"/>
-      <c r="B12" s="6"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="8"/>
-      <c r="G12" s="10"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="B13" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="C13" s="13" t="n">
-        <v>2000</v>
-      </c>
-      <c r="D13" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" s="14" t="n">
-        <f aca="false">C13*D13</f>
-        <v>2000</v>
-      </c>
-      <c r="F13" s="9"/>
-      <c r="G13" s="10"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5"/>
-      <c r="B14" s="15"/>
-      <c r="C14" s="16"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="10"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="1"/>
-      <c r="B15" s="19" t="s">
-        <v>11</v>
-      </c>
-      <c r="C15" s="20"/>
-      <c r="D15" s="21"/>
-      <c r="E15" s="2" t="n">
-        <f aca="false">SUM(E2:E14)</f>
-        <v>2070</v>
-      </c>
-      <c r="F15" s="22"/>
-      <c r="G15" s="23"/>
-    </row>
+      <c r="A12" s="1"/>
+      <c r="B12" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="20"/>
+      <c r="D12" s="21"/>
+      <c r="E12" s="2" t="n">
+        <f aca="false">SUM(E2:E11)</f>
+        <v>2823</v>
+      </c>
+      <c r="F12" s="22"/>
+      <c r="G12" s="23"/>
+    </row>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Started rc rover Programming
</commit_message>
<xml_diff>
--- a/keyboard_emulator/BOM.xlsx
+++ b/keyboard_emulator/BOM.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -47,9 +47,6 @@
   </si>
   <si>
     <t xml:space="preserve">Arduino Pro Micro</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pin Headers</t>
   </si>
   <si>
     <t xml:space="preserve">Spring Terminal – 4Pin</t>
@@ -87,6 +84,7 @@
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -109,12 +107,14 @@
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -355,7 +355,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -413,7 +413,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G1048576"/>
-  <sheetFormatPr defaultColWidth="10.55078125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.55859375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
@@ -489,144 +489,124 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>9</v>
       </c>
       <c r="C4" s="7" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D4" s="5" t="n">
         <v>2</v>
       </c>
       <c r="E4" s="8" t="n">
         <f aca="false">C4*D4</f>
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F4" s="9"/>
       <c r="G4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>10</v>
       </c>
       <c r="C5" s="7" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E5" s="8" t="n">
         <f aca="false">C5*D5</f>
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="F5" s="9"/>
       <c r="G5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="D6" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="E6" s="8" t="n">
-        <f aca="false">C6*D6</f>
-        <v>28</v>
-      </c>
+      <c r="A6" s="5"/>
+      <c r="B6" s="6"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="8"/>
       <c r="F6" s="9"/>
       <c r="G6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5"/>
-      <c r="B7" s="6"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="8"/>
+      <c r="A7" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>70</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" s="8" t="n">
+        <f aca="false">C7*D7</f>
+        <v>140</v>
+      </c>
       <c r="F7" s="9"/>
       <c r="G7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" s="6" t="s">
+      <c r="A8" s="5"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="8"/>
+      <c r="G8" s="10"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="7" t="n">
-        <v>70</v>
-      </c>
-      <c r="D8" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="E8" s="8" t="n">
-        <f aca="false">C8*D8</f>
-        <v>140</v>
-      </c>
-      <c r="F8" s="9"/>
-      <c r="G8" s="10"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5"/>
-      <c r="B9" s="6"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="8"/>
+      <c r="B9" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="13" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D9" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="14" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F9" s="9"/>
       <c r="G9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="C10" s="13" t="n">
-        <v>2000</v>
-      </c>
-      <c r="D10" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E10" s="14" t="n">
-        <f aca="false">C10*D10</f>
-        <v>2000</v>
-      </c>
+      <c r="A10" s="5"/>
+      <c r="B10" s="15"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="18"/>
       <c r="F10" s="9"/>
       <c r="G10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5"/>
-      <c r="B11" s="15"/>
-      <c r="C11" s="16"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="10"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1"/>
-      <c r="B12" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12" s="20"/>
-      <c r="D12" s="21"/>
-      <c r="E12" s="2" t="n">
-        <f aca="false">SUM(E2:E11)</f>
-        <v>2823</v>
-      </c>
-      <c r="F12" s="22"/>
-      <c r="G12" s="23"/>
-    </row>
+      <c r="A11" s="1"/>
+      <c r="B11" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="20"/>
+      <c r="D11" s="21"/>
+      <c r="E11" s="2" t="n">
+        <f aca="false">SUM(E2:E10)</f>
+        <v>2313</v>
+      </c>
+      <c r="F11" s="22"/>
+      <c r="G11" s="23"/>
+    </row>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>